<commit_message>
February 11 2025 V2
</commit_message>
<xml_diff>
--- a/_downloads/fea83e0df67d4b4d485143ef59be81b3/Indicadores Supermercados la Vaquita 2020-2023.xlsx
+++ b/_downloads/fea83e0df67d4b4d485143ef59be81b3/Indicadores Supermercados la Vaquita 2020-2023.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\ADMINISTRACIÓN FINANCIERA\Examen validación\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\ADMINISTRACIÓN FINANCIERA\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED97AF44-62FD-43E0-A52F-47738BB250E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95081972-638E-4083-BDFC-B1F7E8DADF32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1831C0EF-C4ED-498F-B252-8F4DD8980456}"/>
   </bookViews>
@@ -510,7 +510,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -630,12 +630,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2887,16 +2881,16 @@
         <v>66</v>
       </c>
       <c r="C71" s="13">
-        <f>+C66+C63-C69</f>
-        <v>11.145096568487087</v>
+        <f t="shared" ref="C71:D71" si="32">+C66+C63-C70</f>
+        <v>11.99850202109387</v>
       </c>
       <c r="D71" s="13">
-        <f>+D66+D63-D69</f>
-        <v>16.389279174300093</v>
+        <f t="shared" si="32"/>
+        <v>19.997719563654766</v>
       </c>
       <c r="E71" s="13">
-        <f>+E66+E63-E69</f>
-        <v>34.080779615530787</v>
+        <f>+E66+E63-E70</f>
+        <v>16.508156113455431</v>
       </c>
       <c r="F71" s="4" t="s">
         <v>64</v>
@@ -2954,27 +2948,27 @@
         <v>25005720</v>
       </c>
       <c r="C75" s="29">
-        <f t="shared" ref="C75:E75" si="32">+C11+C13</f>
+        <f t="shared" ref="C75:E75" si="33">+C11+C13</f>
         <v>34196311</v>
       </c>
       <c r="D75" s="16">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>40985288</v>
       </c>
       <c r="E75" s="16">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>65708376</v>
       </c>
       <c r="F75" s="14">
-        <f t="shared" ref="F75:H75" si="33">+C75/B75-1</f>
+        <f t="shared" ref="F75:H75" si="34">+C75/B75-1</f>
         <v>0.36753954695165736</v>
       </c>
       <c r="G75" s="14">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>0.1985295138999057</v>
       </c>
       <c r="H75" s="14">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>0.60321859882990214</v>
       </c>
     </row>
@@ -2987,27 +2981,27 @@
         <v>30882872</v>
       </c>
       <c r="C76" s="16">
-        <f t="shared" ref="C76:E76" si="34">+C45+C46+C47</f>
+        <f t="shared" ref="C76:E76" si="35">+C45+C46+C47</f>
         <v>33435897</v>
       </c>
       <c r="D76" s="16">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>51976223</v>
       </c>
       <c r="E76" s="16">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>66385973</v>
       </c>
       <c r="F76" s="14">
-        <f t="shared" ref="F76" si="35">+C76/B76-1</f>
+        <f t="shared" ref="F76" si="36">+C76/B76-1</f>
         <v>8.2667991500272375E-2</v>
       </c>
       <c r="G76" s="14">
-        <f t="shared" ref="G76" si="36">+D76/C76-1</f>
+        <f t="shared" ref="G76" si="37">+D76/C76-1</f>
         <v>0.55450362225963312</v>
       </c>
       <c r="H76" s="14">
-        <f t="shared" ref="H76" si="37">+E76/D76-1</f>
+        <f t="shared" ref="H76" si="38">+E76/D76-1</f>
         <v>0.27723734369848296</v>
       </c>
     </row>
@@ -3032,15 +3026,15 @@
         <v>16775593</v>
       </c>
       <c r="F77" s="14">
-        <f t="shared" ref="F77:F94" si="38">+C77/B77-1</f>
+        <f t="shared" ref="F77:F94" si="39">+C77/B77-1</f>
         <v>3.2980419386661346</v>
       </c>
       <c r="G77" s="14">
-        <f t="shared" ref="G77:G99" si="39">+D77/C77-1</f>
+        <f t="shared" ref="G77:G99" si="40">+D77/C77-1</f>
         <v>0.66366242770423622</v>
       </c>
       <c r="H77" s="14">
-        <f t="shared" ref="H77:H99" si="40">+E77/D77-1</f>
+        <f t="shared" ref="H77:H99" si="41">+E77/D77-1</f>
         <v>-0.5090353185018951</v>
       </c>
     </row>
@@ -3054,20 +3048,20 @@
         <v>12658352</v>
       </c>
       <c r="D78" s="16">
-        <f t="shared" ref="D78:E78" si="41">+AVERAGE(C77:D77)</f>
+        <f t="shared" ref="D78:E78" si="42">+AVERAGE(C77:D77)</f>
         <v>27353418.5</v>
       </c>
       <c r="E78" s="16">
-        <f t="shared" si="41"/>
+        <f t="shared" si="42"/>
         <v>25472114</v>
       </c>
       <c r="F78" s="14"/>
       <c r="G78" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>1.1608988674039087</v>
       </c>
       <c r="H78" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>-6.8777673986160082E-2</v>
       </c>
     </row>
@@ -3081,20 +3075,20 @@
         <v>24.356281607589992</v>
       </c>
       <c r="D79" s="17">
-        <f t="shared" ref="D79:E79" si="42">+D41/D78</f>
+        <f t="shared" ref="D79:E79" si="43">+D41/D78</f>
         <v>16.59231912822889</v>
       </c>
       <c r="E79" s="17">
-        <f t="shared" si="42"/>
+        <f t="shared" si="43"/>
         <v>21.529222505835204</v>
       </c>
       <c r="F79" s="14"/>
       <c r="G79" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>-0.31876632913218028</v>
       </c>
       <c r="H79" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>0.29754149130407259</v>
       </c>
     </row>
@@ -3111,23 +3105,23 @@
         <v>1.9258714603898566</v>
       </c>
       <c r="D80" s="31">
-        <f t="shared" ref="D80:E80" si="43">+D10/D25</f>
+        <f t="shared" ref="D80:E80" si="44">+D10/D25</f>
         <v>2.0877509448084894</v>
       </c>
       <c r="E80" s="31">
-        <f t="shared" si="43"/>
+        <f t="shared" si="44"/>
         <v>1.2325338430128656</v>
       </c>
       <c r="F80" s="14">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>0.52813071344337303</v>
       </c>
       <c r="G80" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>8.4055186313350072E-2</v>
       </c>
       <c r="H80" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>-0.40963559562612162</v>
       </c>
     </row>
@@ -3140,27 +3134,27 @@
         <v>0.45352384146071567</v>
       </c>
       <c r="C81" s="31">
-        <f t="shared" ref="C81:E81" si="44">+C30/C18</f>
+        <f t="shared" ref="C81:E81" si="45">+C30/C18</f>
         <v>0.46084487185162393</v>
       </c>
       <c r="D81" s="31">
-        <f t="shared" si="44"/>
+        <f t="shared" si="45"/>
         <v>0.45747553788100909</v>
       </c>
       <c r="E81" s="31">
-        <f t="shared" si="44"/>
+        <f t="shared" si="45"/>
         <v>0.59049511285899003</v>
       </c>
       <c r="F81" s="14">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>1.6142548024219883E-2</v>
       </c>
       <c r="G81" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>-7.3112107271091631E-3</v>
       </c>
       <c r="H81" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>0.290768716496006</v>
       </c>
     </row>
@@ -3174,20 +3168,20 @@
         <v>36820083</v>
       </c>
       <c r="D82" s="16">
-        <f t="shared" ref="D82:E82" si="45">+AVERAGE(C30:D30)</f>
+        <f t="shared" ref="D82:E82" si="46">+AVERAGE(C30:D30)</f>
         <v>48200427.5</v>
       </c>
       <c r="E82" s="16">
-        <f t="shared" si="45"/>
+        <f t="shared" si="46"/>
         <v>80169126</v>
       </c>
       <c r="F82" s="14"/>
       <c r="G82" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>0.3090798165772739</v>
       </c>
       <c r="H82" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>0.66324512370766842</v>
       </c>
     </row>
@@ -3201,20 +3195,20 @@
         <v>43593296.5</v>
       </c>
       <c r="D83" s="16">
-        <f t="shared" ref="D83:E83" si="46">+AVERAGE(C36:D36)</f>
+        <f t="shared" ref="D83:E83" si="47">+AVERAGE(C36:D36)</f>
         <v>56808524.5</v>
       </c>
       <c r="E83" s="16">
-        <f t="shared" si="46"/>
+        <f t="shared" si="47"/>
         <v>68460987</v>
       </c>
       <c r="F83" s="14"/>
       <c r="G83" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>0.30314816866395966</v>
       </c>
       <c r="H83" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>0.20511820369494016</v>
       </c>
     </row>
@@ -3228,20 +3222,20 @@
         <v>0.84462717794237008</v>
       </c>
       <c r="D84" s="32">
-        <f t="shared" ref="D84:E84" si="47">+D82/D83</f>
+        <f t="shared" ref="D84:E84" si="48">+D82/D83</f>
         <v>0.8484717377230947</v>
       </c>
       <c r="E84" s="32">
-        <f t="shared" si="47"/>
+        <f t="shared" si="48"/>
         <v>1.1710191382429236</v>
       </c>
       <c r="F84" s="14"/>
       <c r="G84" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>4.5517831785741869E-3</v>
       </c>
       <c r="H84" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>0.38015102469458406</v>
       </c>
     </row>
@@ -3254,27 +3248,27 @@
         <v>2891191</v>
       </c>
       <c r="C85" s="29">
-        <f t="shared" ref="C85:E85" si="48">+C23</f>
+        <f t="shared" ref="C85:E85" si="49">+C23</f>
         <v>3292828</v>
       </c>
       <c r="D85" s="16">
-        <f t="shared" si="48"/>
+        <f t="shared" si="49"/>
         <v>3944110</v>
       </c>
       <c r="E85" s="16">
-        <f t="shared" si="48"/>
+        <f t="shared" si="49"/>
         <v>10703413</v>
       </c>
       <c r="F85" s="14">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>0.13891749109622986</v>
       </c>
       <c r="G85" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>0.19778804116097159</v>
       </c>
       <c r="H85" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>1.7137714211824719</v>
       </c>
     </row>
@@ -3287,27 +3281,27 @@
         <v>8893367</v>
       </c>
       <c r="C86" s="29">
-        <f t="shared" ref="C86:E86" si="49">+C28</f>
+        <f t="shared" ref="C86:E86" si="50">+C28</f>
         <v>16646685</v>
       </c>
       <c r="D86" s="16">
-        <f t="shared" si="49"/>
+        <f t="shared" si="50"/>
         <v>16100930</v>
       </c>
       <c r="E86" s="16">
-        <f t="shared" si="49"/>
+        <f t="shared" si="50"/>
         <v>30627239</v>
       </c>
       <c r="F86" s="14">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>0.8718090684889086</v>
       </c>
       <c r="G86" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>-3.2784605463490157E-2</v>
       </c>
       <c r="H86" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>0.9022031025537034</v>
       </c>
     </row>
@@ -3320,27 +3314,27 @@
         <v>11784558</v>
       </c>
       <c r="C87" s="33">
-        <f t="shared" ref="C87:E87" si="50">SUM(C85:C86)</f>
+        <f t="shared" ref="C87:E87" si="51">SUM(C85:C86)</f>
         <v>19939513</v>
       </c>
       <c r="D87" s="20">
-        <f t="shared" si="50"/>
+        <f t="shared" si="51"/>
         <v>20045040</v>
       </c>
       <c r="E87" s="20">
-        <f t="shared" si="50"/>
+        <f t="shared" si="51"/>
         <v>41330652</v>
       </c>
       <c r="F87" s="36">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>0.6920034675886868</v>
       </c>
       <c r="G87" s="24">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>5.2923559366770956E-3</v>
       </c>
       <c r="H87" s="24">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>1.0618892254642547</v>
       </c>
     </row>
@@ -3353,27 +3347,27 @@
         <v>1046763</v>
       </c>
       <c r="C88" s="29">
-        <f t="shared" ref="C88:E88" si="51">+C51</f>
+        <f t="shared" ref="C88:E88" si="52">+C51</f>
         <v>784519</v>
       </c>
       <c r="D88" s="16">
-        <f t="shared" si="51"/>
+        <f t="shared" si="52"/>
         <v>1987404</v>
       </c>
       <c r="E88" s="16">
-        <f t="shared" si="51"/>
+        <f t="shared" si="52"/>
         <v>4416288</v>
       </c>
       <c r="F88" s="14">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>-0.25052853415720655</v>
       </c>
       <c r="G88" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>1.5332770780567455</v>
       </c>
       <c r="H88" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>1.22213903162115</v>
       </c>
     </row>
@@ -3386,11 +3380,11 @@
         <v>16.702867793378253</v>
       </c>
       <c r="C89" s="30">
-        <f t="shared" ref="C89:D89" si="52">+C58/C88</f>
+        <f t="shared" ref="C89:D89" si="53">+C58/C88</f>
         <v>25.098225791854627</v>
       </c>
       <c r="D89" s="30">
-        <f t="shared" si="52"/>
+        <f t="shared" si="53"/>
         <v>12.059273303263957</v>
       </c>
       <c r="E89" s="30">
@@ -3398,15 +3392,15 @@
         <v>6.1827355915193936</v>
       </c>
       <c r="F89" s="14">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>0.50262973414689061</v>
       </c>
       <c r="G89" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>-0.51951690118360194</v>
       </c>
       <c r="H89" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>-0.48730446387296178</v>
       </c>
     </row>
@@ -3419,27 +3413,27 @@
         <v>3.8509879005026422E-3</v>
       </c>
       <c r="C90" s="34">
-        <f t="shared" ref="C90:E90" si="53">+C88/C41</f>
+        <f t="shared" ref="C90:E90" si="54">+C88/C41</f>
         <v>2.5445753228695968E-3</v>
       </c>
       <c r="D90" s="21">
-        <f t="shared" si="53"/>
+        <f t="shared" si="54"/>
         <v>4.3789245004538868E-3</v>
       </c>
       <c r="E90" s="21">
-        <f t="shared" si="53"/>
+        <f t="shared" si="54"/>
         <v>8.0531177893532584E-3</v>
       </c>
       <c r="F90" s="14">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>-0.33924089386583856</v>
       </c>
       <c r="G90" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>0.7208861773899613</v>
       </c>
       <c r="H90" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>0.83906294536901282</v>
       </c>
     </row>
@@ -3447,32 +3441,32 @@
       <c r="A91" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B91" s="43">
+      <c r="B91" s="39">
         <f>+B43/B41</f>
         <v>0.17201448287516471</v>
       </c>
-      <c r="C91" s="44">
-        <f t="shared" ref="C91:E91" si="54">+C43/C41</f>
+      <c r="C91" s="40">
+        <f t="shared" ref="C91:E91" si="55">+C43/C41</f>
         <v>0.16574484130417844</v>
       </c>
-      <c r="D91" s="43">
-        <f t="shared" si="54"/>
+      <c r="D91" s="39">
+        <f t="shared" si="55"/>
         <v>0.16205743413048468</v>
       </c>
-      <c r="E91" s="43">
-        <f t="shared" si="54"/>
+      <c r="E91" s="39">
+        <f t="shared" si="55"/>
         <v>0.16500005534333922</v>
       </c>
       <c r="F91" s="14">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>-3.6448335431943368E-2</v>
       </c>
       <c r="G91" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>-2.2247492861189877E-2</v>
       </c>
       <c r="H91" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>1.8157890927023024E-2</v>
       </c>
     </row>
@@ -3485,27 +3479,27 @@
         <v>6.0015908659284738E-2</v>
       </c>
       <c r="C92" s="34">
-        <f t="shared" ref="C92:E92" si="55">+C49/C41</f>
+        <f t="shared" ref="C92:E92" si="56">+C49/C41</f>
         <v>5.9903580413278715E-2</v>
       </c>
       <c r="D92" s="21">
-        <f t="shared" si="55"/>
+        <f t="shared" si="56"/>
         <v>4.9159191672434877E-2</v>
       </c>
       <c r="E92" s="21">
-        <f t="shared" si="55"/>
+        <f t="shared" si="56"/>
         <v>4.5790732410469021E-2</v>
       </c>
       <c r="F92" s="14">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>-1.8716411784035492E-3</v>
       </c>
       <c r="G92" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>-0.17936137818002862</v>
       </c>
       <c r="H92" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>-6.852145341223459E-2</v>
       </c>
     </row>
@@ -3518,27 +3512,27 @@
         <v>6.4322541775994918E-2</v>
       </c>
       <c r="C93" s="34">
-        <f t="shared" ref="C93:E93" si="56">+C58/C41</f>
+        <f t="shared" ref="C93:E93" si="57">+C58/C41</f>
         <v>6.3864325997762525E-2</v>
       </c>
       <c r="D93" s="21">
-        <f t="shared" si="56"/>
+        <f t="shared" si="57"/>
         <v>5.280664732533201E-2</v>
       </c>
       <c r="E93" s="21">
-        <f t="shared" si="56"/>
+        <f t="shared" si="57"/>
         <v>4.979029797893237E-2</v>
       </c>
       <c r="F93" s="14">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>-7.1237200144879109E-3</v>
       </c>
       <c r="G93" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>-0.17314327677736585</v>
       </c>
       <c r="H93" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>-5.7120637252663808E-2</v>
       </c>
     </row>
@@ -3551,27 +3545,27 @@
         <v>3.9617180171820615E-2</v>
       </c>
       <c r="C94" s="34">
-        <f t="shared" ref="C94:E94" si="57">+C54/C41</f>
+        <f t="shared" ref="C94:E94" si="58">+C54/C41</f>
         <v>4.0239961296665495E-2</v>
       </c>
       <c r="D94" s="21">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>2.9759665369582369E-2</v>
       </c>
       <c r="E94" s="21">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>2.3698521143918194E-2</v>
       </c>
       <c r="F94" s="14">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>1.5719976084715315E-2</v>
       </c>
       <c r="G94" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>-0.26044498029752283</v>
       </c>
       <c r="H94" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>-0.20366977082542492</v>
       </c>
     </row>
@@ -3585,20 +3579,20 @@
         <v>80413379.5</v>
       </c>
       <c r="D95" s="16">
-        <f t="shared" ref="D95:E95" si="58">+AVERAGE(C18:D18)</f>
+        <f t="shared" ref="D95:E95" si="59">+AVERAGE(C18:D18)</f>
         <v>105008952</v>
       </c>
       <c r="E95" s="16">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>148630113</v>
       </c>
       <c r="F95" s="14"/>
       <c r="G95" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>0.30586418146995054</v>
       </c>
       <c r="H95" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>0.41540421239514891</v>
       </c>
     </row>
@@ -3612,20 +3606,20 @@
         <v>3.8340682597477449</v>
       </c>
       <c r="D96" s="34">
-        <f t="shared" ref="D96:E96" si="59">+D41/D95</f>
+        <f t="shared" ref="D96:E96" si="60">+D41/D95</f>
         <v>4.3220757883575489</v>
       </c>
       <c r="E96" s="34">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>3.6896615290873123</v>
       </c>
       <c r="F96" s="14"/>
       <c r="G96" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>0.12728190933197192</v>
       </c>
       <c r="H96" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>-0.14632188102156418</v>
       </c>
     </row>
@@ -3639,20 +3633,20 @@
         <v>0.1542827583810229</v>
       </c>
       <c r="D97" s="34">
-        <f t="shared" ref="D97:E97" si="60">+D54/D95</f>
+        <f t="shared" ref="D97:E97" si="61">+D54/D95</f>
         <v>0.12862352916349457</v>
       </c>
       <c r="E97" s="34">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>8.7439521760977204E-2</v>
       </c>
       <c r="F97" s="14"/>
       <c r="G97" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>-0.16631300533374749</v>
       </c>
       <c r="H97" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>-0.32019030787258207</v>
       </c>
     </row>
@@ -3666,20 +3660,20 @@
         <v>0.22967441630779864</v>
       </c>
       <c r="D98" s="34">
-        <f t="shared" ref="D98:E98" si="61">+D49/D95</f>
+        <f t="shared" ref="D98:E98" si="62">+D49/D95</f>
         <v>0.21246975210265884</v>
       </c>
       <c r="E98" s="34">
-        <f t="shared" si="61"/>
+        <f t="shared" si="62"/>
         <v>0.16895230376363907</v>
       </c>
       <c r="F98" s="14"/>
       <c r="G98" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>-7.4908927523224644E-2</v>
       </c>
       <c r="H98" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>-0.20481714648018923</v>
       </c>
     </row>
@@ -3693,20 +3687,20 @@
         <v>0.28459416919755082</v>
       </c>
       <c r="D99" s="34">
-        <f t="shared" ref="D99:E99" si="62">+D54/D83</f>
+        <f t="shared" ref="D99:E99" si="63">+D54/D83</f>
         <v>0.23775695846492192</v>
       </c>
       <c r="E99" s="34">
-        <f t="shared" si="62"/>
+        <f t="shared" si="63"/>
         <v>0.1898328751818901</v>
       </c>
       <c r="F99" s="14"/>
       <c r="G99" s="14">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>-0.16457544040586747</v>
       </c>
       <c r="H99" s="14">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>-0.20156753178730802</v>
       </c>
     </row>
@@ -3729,20 +3723,20 @@
         <v>4.0239961296665495E-2</v>
       </c>
       <c r="D101" s="21">
-        <f t="shared" ref="D101:E101" si="63">+D94</f>
+        <f t="shared" ref="D101:E101" si="64">+D94</f>
         <v>2.9759665369582369E-2</v>
       </c>
       <c r="E101" s="21">
-        <f t="shared" si="63"/>
+        <f t="shared" si="64"/>
         <v>2.3698521143918194E-2</v>
       </c>
       <c r="F101" s="14"/>
       <c r="G101" s="14">
-        <f t="shared" ref="G101:G104" si="64">+D101/C101-1</f>
+        <f t="shared" ref="G101:G104" si="65">+D101/C101-1</f>
         <v>-0.26044498029752283</v>
       </c>
       <c r="H101" s="14">
-        <f t="shared" ref="H101:H104" si="65">+E101/D101-1</f>
+        <f t="shared" ref="H101:H104" si="66">+E101/D101-1</f>
         <v>-0.20366977082542492</v>
       </c>
     </row>
@@ -3756,20 +3750,20 @@
         <v>3.8340682597477449</v>
       </c>
       <c r="D102" s="18">
-        <f t="shared" ref="D102:E102" si="66">+D96</f>
+        <f t="shared" ref="D102:E102" si="67">+D96</f>
         <v>4.3220757883575489</v>
       </c>
       <c r="E102" s="18">
-        <f t="shared" si="66"/>
+        <f t="shared" si="67"/>
         <v>3.6896615290873123</v>
       </c>
       <c r="F102" s="14"/>
       <c r="G102" s="14">
-        <f t="shared" si="64"/>
+        <f t="shared" si="65"/>
         <v>0.12728190933197192</v>
       </c>
       <c r="H102" s="14">
-        <f t="shared" si="65"/>
+        <f t="shared" si="66"/>
         <v>-0.14632188102156418</v>
       </c>
     </row>
@@ -3783,20 +3777,20 @@
         <v>1.8446271779423702</v>
       </c>
       <c r="D103" s="19">
-        <f t="shared" ref="D103:E103" si="67">+D95/D83</f>
+        <f t="shared" ref="D103:E103" si="68">+D95/D83</f>
         <v>1.8484717377230948</v>
       </c>
       <c r="E103" s="19">
-        <f t="shared" si="67"/>
+        <f t="shared" si="68"/>
         <v>2.1710191382429236</v>
       </c>
       <c r="F103" s="14"/>
       <c r="G103" s="14">
-        <f t="shared" si="64"/>
+        <f t="shared" si="65"/>
         <v>2.084193395119005E-3</v>
       </c>
       <c r="H103" s="14">
-        <f t="shared" si="65"/>
+        <f t="shared" si="66"/>
         <v>0.17449409365443436</v>
       </c>
     </row>
@@ -3810,20 +3804,20 @@
         <v>0.28459416919755076</v>
       </c>
       <c r="D104" s="28">
-        <f t="shared" ref="D104:E104" si="68">+D101*D102*D103</f>
+        <f t="shared" ref="D104:E104" si="69">+D101*D102*D103</f>
         <v>0.23775695846492195</v>
       </c>
       <c r="E104" s="28">
-        <f t="shared" si="68"/>
+        <f t="shared" si="69"/>
         <v>0.1898328751818901</v>
       </c>
       <c r="F104" s="25"/>
       <c r="G104" s="23">
-        <f t="shared" si="64"/>
+        <f t="shared" si="65"/>
         <v>-0.16457544040586725</v>
       </c>
       <c r="H104" s="23">
-        <f t="shared" si="65"/>
+        <f t="shared" si="66"/>
         <v>-0.20156753178730813</v>
       </c>
     </row>
@@ -3834,11 +3828,11 @@
         <v>1</v>
       </c>
       <c r="D105" s="35" t="b">
-        <f t="shared" ref="D105:E105" si="69">+D104=D99</f>
+        <f t="shared" ref="D105:E105" si="70">+D104=D99</f>
         <v>1</v>
       </c>
       <c r="E105" s="35" t="b">
-        <f t="shared" si="69"/>
+        <f t="shared" si="70"/>
         <v>1</v>
       </c>
     </row>
@@ -3905,11 +3899,11 @@
         <v>0.1342582476504226</v>
       </c>
       <c r="D110" s="34">
-        <f t="shared" ref="D110:E110" si="70">+H41</f>
+        <f t="shared" ref="D110:E110" si="71">+H41</f>
         <v>0.47207706781567849</v>
       </c>
       <c r="E110" s="34">
-        <f t="shared" si="70"/>
+        <f t="shared" si="71"/>
         <v>0.20829960563164507</v>
       </c>
     </row>
@@ -3923,11 +3917,11 @@
         <v>0.14284703636063734</v>
       </c>
       <c r="D111" s="34">
-        <f t="shared" ref="D111:E111" si="71">+H42</f>
+        <f t="shared" ref="D111:E111" si="72">+H42</f>
         <v>0.47858364734774805</v>
       </c>
       <c r="E111" s="34">
-        <f t="shared" si="71"/>
+        <f t="shared" si="72"/>
         <v>0.20405639351205807</v>
       </c>
     </row>
@@ -3941,11 +3935,11 @@
         <v>8.2667991500272375E-2</v>
       </c>
       <c r="D112" s="34">
-        <f t="shared" ref="D112:E112" si="72">+G76</f>
+        <f t="shared" ref="D112:E112" si="73">+G76</f>
         <v>0.55450362225963312</v>
       </c>
       <c r="E112" s="34">
-        <f t="shared" si="72"/>
+        <f t="shared" si="73"/>
         <v>0.27723734369848296</v>
       </c>
     </row>
@@ -3959,11 +3953,11 @@
         <v>-3.6448335431943368E-2</v>
       </c>
       <c r="D113" s="34">
-        <f t="shared" ref="D113:E113" si="73">+G91</f>
+        <f t="shared" ref="D113:E113" si="74">+G91</f>
         <v>-2.2247492861189877E-2</v>
       </c>
       <c r="E113" s="34">
-        <f t="shared" si="73"/>
+        <f t="shared" si="74"/>
         <v>1.8157890927023024E-2</v>
       </c>
     </row>
@@ -3977,11 +3971,11 @@
         <v>-7.1237200144879109E-3</v>
       </c>
       <c r="D114" s="34">
-        <f t="shared" ref="D114:E114" si="74">+G93</f>
+        <f t="shared" ref="D114:E114" si="75">+G93</f>
         <v>-0.17314327677736585</v>
       </c>
       <c r="E114" s="34">
-        <f t="shared" si="74"/>
+        <f t="shared" si="75"/>
         <v>-5.7120637252663808E-2</v>
       </c>
     </row>
@@ -3995,11 +3989,11 @@
         <v>1.5719976084715315E-2</v>
       </c>
       <c r="D115" s="34">
-        <f t="shared" ref="D115:E115" si="75">+G94</f>
+        <f t="shared" ref="D115:E115" si="76">+G94</f>
         <v>-0.26044498029752283</v>
       </c>
       <c r="E115" s="34">
-        <f t="shared" si="75"/>
+        <f t="shared" si="76"/>
         <v>-0.20366977082542492</v>
       </c>
     </row>
@@ -4013,11 +4007,11 @@
         <v>0.6920034675886868</v>
       </c>
       <c r="D116" s="40">
-        <f t="shared" ref="D116:E116" si="76">+G87</f>
+        <f t="shared" ref="D116:E116" si="77">+G87</f>
         <v>5.2923559366770956E-3</v>
       </c>
       <c r="E116" s="40">
-        <f t="shared" si="76"/>
+        <f t="shared" si="77"/>
         <v>1.0618892254642547</v>
       </c>
     </row>

</xml_diff>